<commit_message>
[chore] SupportItem 데이터에 ItemCategory, HealAmount 필드 및 회복 아이템 추가
회복 아이템은 대응페널티 빈 값으로 둬도 됩니다.
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/SupportItem.xlsx
+++ b/JsonConverter/ExcelFiles/SupportItem.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GameProjects\ACE\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FF55CD-8F83-47BF-9715-287323E0A2F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{592D079C-99FC-4A7B-A683-C22C3AB20C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1605" yWindow="1245" windowWidth="24480" windowHeight="13095" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-180" yWindow="465" windowWidth="24480" windowHeight="14130" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SupportItem" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="48">
   <si>
     <t>아이템ID</t>
   </si>
@@ -190,6 +190,71 @@
   </si>
   <si>
     <t>StockCount</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>아이템 종류</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>string</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>ItemCategory</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>HealAmount</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>회복량</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>int</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Penalty</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>item_03</t>
+  </si>
+  <si>
+    <t>비타민음료</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vitamin Drink</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Heal</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>맛있는 비타민 음료다.
+영웅들의 삶의 희망!</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>item_04</t>
+  </si>
+  <si>
+    <t>반창고</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>BandAid</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>영웅들이 아야!했나보다.
+영웅일지라도 다친 살갗은 아픈 법이다.
+그들의 아코!한 살갗을 덮어 위로해주자.</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -602,22 +667,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R1000"/>
+  <dimension ref="A1:T1000"/>
   <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.875" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="17.125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="5.25" style="1" customWidth="1"/>
-    <col min="9" max="9" width="24.375" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="11.5" style="3"/>
+    <col min="3" max="4" width="17.125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="17.875" style="1" customWidth="1"/>
+    <col min="6" max="7" width="18" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="10.375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="5.25" style="1" customWidth="1"/>
+    <col min="11" max="11" width="24.375" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="11.5" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" customHeight="1">
+    <row r="1" spans="1:20" ht="15.75" customHeight="1">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -628,25 +693,31 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="12.75">
+    <row r="2" spans="1:20" ht="12.75">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -657,25 +728,31 @@
         <v>9</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:18" s="10" customFormat="1" ht="15.75" customHeight="1">
+    <row r="3" spans="1:20" s="10" customFormat="1" ht="15.75" customHeight="1">
       <c r="A3" s="7" t="s">
         <v>11</v>
       </c>
@@ -686,25 +763,31 @@
         <v>27</v>
       </c>
       <c r="D3" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="G3" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="I3" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="J3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="K3" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="108">
+    <row r="4" spans="1:20" ht="108">
       <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
@@ -715,25 +798,29 @@
         <v>16</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="1">
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1">
         <v>1</v>
       </c>
-      <c r="G4" s="11">
+      <c r="I4" s="11">
         <v>2</v>
       </c>
-      <c r="H4" s="11">
+      <c r="J4" s="11">
         <v>100</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="K4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
       <c r="L4" s="13"/>
       <c r="M4" s="13"/>
       <c r="N4" s="13"/>
@@ -741,8 +828,10 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="13"/>
       <c r="R4" s="13"/>
-    </row>
-    <row r="5" spans="1:18" ht="63.75">
+      <c r="S4" s="13"/>
+      <c r="T4" s="13"/>
+    </row>
+    <row r="5" spans="1:20" ht="63.75">
       <c r="A5" s="4" t="s">
         <v>19</v>
       </c>
@@ -753,25 +842,29 @@
         <v>21</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F5" s="1">
+      <c r="G5" s="4">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
         <v>2</v>
       </c>
-      <c r="G5" s="11">
+      <c r="I5" s="11">
         <v>2</v>
       </c>
-      <c r="H5" s="11">
+      <c r="J5" s="11">
         <v>150</v>
       </c>
-      <c r="I5" s="14" t="s">
+      <c r="K5" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
       <c r="L5" s="13"/>
       <c r="M5" s="13"/>
       <c r="N5" s="13"/>
@@ -779,18 +872,39 @@
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
       <c r="R5" s="13"/>
-    </row>
-    <row r="6" spans="1:18" ht="15.75" customHeight="1">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
+      <c r="S5" s="13"/>
+      <c r="T5" s="13"/>
+    </row>
+    <row r="6" spans="1:20" ht="25.5">
+      <c r="A6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="E6" s="4"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4">
+        <v>5</v>
+      </c>
+      <c r="H6" s="1">
+        <v>1</v>
+      </c>
+      <c r="I6" s="15">
+        <v>0</v>
+      </c>
+      <c r="J6" s="15">
+        <v>80</v>
+      </c>
+      <c r="K6" s="14" t="s">
+        <v>43</v>
+      </c>
       <c r="L6" s="13"/>
       <c r="M6" s="13"/>
       <c r="N6" s="13"/>
@@ -798,18 +912,39 @@
       <c r="P6" s="13"/>
       <c r="Q6" s="13"/>
       <c r="R6" s="13"/>
-    </row>
-    <row r="7" spans="1:18" ht="15.75" customHeight="1">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="S6" s="13"/>
+      <c r="T6" s="13"/>
+    </row>
+    <row r="7" spans="1:20" ht="63.75">
+      <c r="A7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>42</v>
+      </c>
       <c r="E7" s="4"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4">
+        <v>10</v>
+      </c>
+      <c r="H7" s="1">
+        <v>1</v>
+      </c>
+      <c r="I7" s="15">
+        <v>0</v>
+      </c>
+      <c r="J7" s="15">
+        <v>50</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>47</v>
+      </c>
       <c r="L7" s="13"/>
       <c r="M7" s="13"/>
       <c r="N7" s="13"/>
@@ -817,18 +952,20 @@
       <c r="P7" s="13"/>
       <c r="Q7" s="13"/>
       <c r="R7" s="13"/>
-    </row>
-    <row r="8" spans="1:18" ht="15.75" customHeight="1">
+      <c r="S7" s="13"/>
+      <c r="T7" s="13"/>
+    </row>
+    <row r="8" spans="1:20" ht="15.75" customHeight="1">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="13"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="16"/>
       <c r="L8" s="13"/>
       <c r="M8" s="13"/>
       <c r="N8" s="13"/>
@@ -836,18 +973,20 @@
       <c r="P8" s="13"/>
       <c r="Q8" s="13"/>
       <c r="R8" s="13"/>
-    </row>
-    <row r="9" spans="1:18" ht="15.75" customHeight="1">
+      <c r="S8" s="13"/>
+      <c r="T8" s="13"/>
+    </row>
+    <row r="9" spans="1:20" ht="15.75" customHeight="1">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="16"/>
       <c r="L9" s="13"/>
       <c r="M9" s="13"/>
       <c r="N9" s="13"/>
@@ -855,18 +994,20 @@
       <c r="P9" s="13"/>
       <c r="Q9" s="13"/>
       <c r="R9" s="13"/>
-    </row>
-    <row r="10" spans="1:18" ht="15.75" customHeight="1">
+      <c r="S9" s="13"/>
+      <c r="T9" s="13"/>
+    </row>
+    <row r="10" spans="1:20" ht="15.75" customHeight="1">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="16"/>
       <c r="L10" s="13"/>
       <c r="M10" s="13"/>
       <c r="N10" s="13"/>
@@ -874,19 +1015,21 @@
       <c r="P10" s="13"/>
       <c r="Q10" s="13"/>
       <c r="R10" s="13"/>
-    </row>
-    <row r="11" spans="1:18" ht="15.75" customHeight="1">
+      <c r="S10" s="13"/>
+      <c r="T10" s="13"/>
+    </row>
+    <row r="11" spans="1:20" ht="15.75" customHeight="1">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
       <c r="H11" s="15"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="16"/>
       <c r="L11" s="13"/>
       <c r="M11" s="13"/>
       <c r="N11" s="13"/>
@@ -894,19 +1037,21 @@
       <c r="P11" s="13"/>
       <c r="Q11" s="13"/>
       <c r="R11" s="13"/>
-    </row>
-    <row r="12" spans="1:18" ht="15.75" customHeight="1">
+      <c r="S11" s="13"/>
+      <c r="T11" s="13"/>
+    </row>
+    <row r="12" spans="1:20" ht="15.75" customHeight="1">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
       <c r="H12" s="15"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="13"/>
-      <c r="K12" s="13"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="16"/>
       <c r="L12" s="13"/>
       <c r="M12" s="13"/>
       <c r="N12" s="13"/>
@@ -914,19 +1059,21 @@
       <c r="P12" s="13"/>
       <c r="Q12" s="13"/>
       <c r="R12" s="13"/>
-    </row>
-    <row r="13" spans="1:18" ht="15.75" customHeight="1">
+      <c r="S12" s="13"/>
+      <c r="T12" s="13"/>
+    </row>
+    <row r="13" spans="1:20" ht="15.75" customHeight="1">
       <c r="A13" s="4"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
       <c r="H13" s="15"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="16"/>
       <c r="L13" s="13"/>
       <c r="M13" s="13"/>
       <c r="N13" s="13"/>
@@ -934,19 +1081,21 @@
       <c r="P13" s="13"/>
       <c r="Q13" s="13"/>
       <c r="R13" s="13"/>
-    </row>
-    <row r="14" spans="1:18" ht="15.75" customHeight="1">
+      <c r="S13" s="13"/>
+      <c r="T13" s="13"/>
+    </row>
+    <row r="14" spans="1:20" ht="15.75" customHeight="1">
       <c r="A14" s="4"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
       <c r="H14" s="15"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="16"/>
       <c r="L14" s="13"/>
       <c r="M14" s="13"/>
       <c r="N14" s="13"/>
@@ -954,19 +1103,21 @@
       <c r="P14" s="13"/>
       <c r="Q14" s="13"/>
       <c r="R14" s="13"/>
-    </row>
-    <row r="15" spans="1:18" ht="15.75" customHeight="1">
+      <c r="S14" s="13"/>
+      <c r="T14" s="13"/>
+    </row>
+    <row r="15" spans="1:20" ht="15.75" customHeight="1">
       <c r="A15" s="4"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
       <c r="H15" s="15"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="13"/>
-      <c r="K15" s="13"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="16"/>
       <c r="L15" s="13"/>
       <c r="M15" s="13"/>
       <c r="N15" s="13"/>
@@ -974,29 +1125,37 @@
       <c r="P15" s="13"/>
       <c r="Q15" s="13"/>
       <c r="R15" s="13"/>
-    </row>
-    <row r="16" spans="1:18" ht="15.75" customHeight="1">
+      <c r="S15" s="13"/>
+      <c r="T15" s="13"/>
+    </row>
+    <row r="16" spans="1:20" ht="15.75" customHeight="1">
       <c r="A16" s="15"/>
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
       <c r="D16" s="15"/>
       <c r="E16" s="15"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+    </row>
+    <row r="17" spans="1:10" ht="15.75" customHeight="1">
       <c r="A17" s="15"/>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
       <c r="E17" s="15"/>
-    </row>
-    <row r="18" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+    </row>
+    <row r="18" spans="1:10" ht="15.75" customHeight="1">
       <c r="A18" s="15"/>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
       <c r="E18" s="15"/>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+    </row>
+    <row r="19" spans="1:10" ht="15.75" customHeight="1">
       <c r="A19" s="15"/>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -1005,140 +1164,174 @@
       <c r="F19" s="15"/>
       <c r="G19" s="15"/>
       <c r="H19" s="15"/>
-    </row>
-    <row r="20" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+    </row>
+    <row r="20" spans="1:10" ht="15.75" customHeight="1">
       <c r="A20" s="15"/>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
       <c r="D20" s="15"/>
       <c r="E20" s="15"/>
-    </row>
-    <row r="21" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+    </row>
+    <row r="21" spans="1:10" ht="15.75" customHeight="1">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
       <c r="D21" s="15"/>
       <c r="E21" s="15"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+    </row>
+    <row r="22" spans="1:10" ht="15.75" customHeight="1">
       <c r="A22" s="15"/>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
       <c r="D22" s="15"/>
       <c r="E22" s="15"/>
-    </row>
-    <row r="23" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+    </row>
+    <row r="23" spans="1:10" ht="15.75" customHeight="1">
       <c r="A23" s="15"/>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
       <c r="D23" s="15"/>
       <c r="E23" s="15"/>
-    </row>
-    <row r="24" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+    </row>
+    <row r="24" spans="1:10" ht="15.75" customHeight="1">
       <c r="A24" s="15"/>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
       <c r="D24" s="15"/>
       <c r="E24" s="15"/>
-    </row>
-    <row r="25" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+    </row>
+    <row r="25" spans="1:10" ht="15.75" customHeight="1">
       <c r="A25" s="15"/>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
       <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-    </row>
-    <row r="26" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+    </row>
+    <row r="26" spans="1:10" ht="15.75" customHeight="1">
       <c r="A26" s="15"/>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
       <c r="D26" s="15"/>
       <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
       <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-    </row>
-    <row r="27" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I26" s="15"/>
+      <c r="J26" s="15"/>
+    </row>
+    <row r="27" spans="1:10" ht="15.75" customHeight="1">
       <c r="A27" s="15"/>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
       <c r="D27" s="15"/>
       <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
       <c r="G27" s="15"/>
-      <c r="H27" s="15"/>
-    </row>
-    <row r="28" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I27" s="15"/>
+      <c r="J27" s="15"/>
+    </row>
+    <row r="28" spans="1:10" ht="15.75" customHeight="1">
       <c r="A28" s="15"/>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
       <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-    </row>
-    <row r="29" spans="1:8" ht="15.75" customHeight="1">
+      <c r="I28" s="15"/>
+      <c r="J28" s="15"/>
+    </row>
+    <row r="29" spans="1:10" ht="15.75" customHeight="1">
       <c r="A29" s="15"/>
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
       <c r="D29" s="15"/>
       <c r="E29" s="15"/>
-    </row>
-    <row r="30" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+    </row>
+    <row r="30" spans="1:10" ht="15.75" customHeight="1">
       <c r="A30" s="15"/>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
       <c r="D30" s="15"/>
       <c r="E30" s="15"/>
-    </row>
-    <row r="31" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+    </row>
+    <row r="31" spans="1:10" ht="15.75" customHeight="1">
       <c r="A31" s="15"/>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
       <c r="D31" s="15"/>
       <c r="E31" s="15"/>
-    </row>
-    <row r="32" spans="1:8" ht="15.75" customHeight="1">
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+    </row>
+    <row r="32" spans="1:10" ht="15.75" customHeight="1">
       <c r="A32" s="15"/>
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
       <c r="D32" s="15"/>
       <c r="E32" s="15"/>
-    </row>
-    <row r="33" spans="1:5" ht="15.75" customHeight="1">
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+    </row>
+    <row r="33" spans="1:7" ht="15.75" customHeight="1">
       <c r="A33" s="15"/>
       <c r="B33" s="15"/>
       <c r="C33" s="15"/>
       <c r="D33" s="15"/>
       <c r="E33" s="15"/>
-    </row>
-    <row r="34" spans="1:5" ht="15.75" customHeight="1">
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+    </row>
+    <row r="34" spans="1:7" ht="15.75" customHeight="1">
       <c r="A34" s="15"/>
       <c r="B34" s="15"/>
       <c r="C34" s="15"/>
       <c r="D34" s="15"/>
       <c r="E34" s="15"/>
-    </row>
-    <row r="35" spans="1:5" ht="15.75" customHeight="1">
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+    </row>
+    <row r="35" spans="1:7" ht="15.75" customHeight="1">
       <c r="A35" s="15"/>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
       <c r="D35" s="15"/>
       <c r="E35" s="15"/>
-    </row>
-    <row r="36" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="37" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="38" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="39" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="40" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="41" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="42" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="43" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="44" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="45" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="46" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="47" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="48" spans="1:5" ht="15.75" customHeight="1"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="37" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="38" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="39" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="40" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="41" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="42" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="43" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="44" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="45" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="46" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="47" spans="1:7" ht="15.75" customHeight="1"/>
+    <row r="48" spans="1:7" ht="15.75" customHeight="1"/>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>

</xml_diff>